<commit_message>
Refinar frontera: 3 DUDA con revisión (TT/DO/CO DNP), 3 confirmados ENTRA
Ajustes según decisiones del equipo:
- TT EngageTT, DO CiudadanIA, CO DNP Diálogos → DUDA con URL para revisar
  (posible IA planeada/usada o módulo de participación). Grupo C nuevo.
- CL La voz de nuevos votantes, CL Jornada UNAB → ENTRA (ejecutados por el equipo).
- CO Chatico → ENTRA (tiene módulos de participación).
- CR U-Report queda DUDA (frontera); BR Colab queda en revisión.

EXCLUIR baja a 4 confirmados (PE conteo, CO Descongestión, BR ParticipACT, CR dIAra).
calc_preliminar: central sube a 39 inic (prom regional 28); rango techo 29 /
central 28 / conservador 24.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/calculo_preliminar_ILIA2026.xlsx
+++ b/data/gates/calculo_preliminar_ILIA2026.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -590,16 +590,16 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>81</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -749,19 +749,19 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Rep. Dominicana</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>26</v>
@@ -773,22 +773,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>1</v>
@@ -797,64 +797,112 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>22</v>
+        <v>6</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>25</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TT</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Trinidad y Tobago</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
           <t>Promedio (países con iniciativas)</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="5" t="n">
-        <v>42</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Promedio regional (20 países, 0 si no hay)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr"/>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="F16" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -867,7 +915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1026,7 +1074,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>75</v>
@@ -1035,16 +1083,16 @@
         <v>67</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>50</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>2</v>
@@ -1290,12 +1338,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Rep. Dominicana</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -1308,13 +1356,13 @@
         <v>67</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>1</v>
@@ -1323,37 +1371,37 @@
         <v>2</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>67</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>1</v>
@@ -1362,25 +1410,25 @@
         <v>2</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>67</v>
@@ -1392,7 +1440,7 @@
         <v>25</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>1</v>
@@ -1401,6 +1449,84 @@
         <v>2</v>
       </c>
       <c r="K13" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TT</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Trinidad y Tobago</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1415,7 +1541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1640,63 +1766,105 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Rep. Dominicana</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>17</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
         <v>12</v>
       </c>
       <c r="D13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TT</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Trinidad y Tobago</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D15" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E15" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1781,13 +1949,13 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -1802,13 +1970,13 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -1859,7 +2027,7 @@
         <v>88</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8">
@@ -1898,10 +2066,10 @@
         <v>81</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>62</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10">
@@ -2033,82 +2201,82 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Rep. Dominicana</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>26</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Trinidad y Tobago</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>0</v>
@@ -2117,22 +2285,22 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Trinidad y Tobago</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -2146,7 +2314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3355,7 +3523,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>ECHO – HáblameD Medellín</t>
+          <t>DNP - Diálogos Regionales Vinculantes (PND 2022-2026)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -3365,12 +3533,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
+          <t>Participación Digital; Mini públicos</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Implementación; Análisis</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
@@ -3378,7 +3546,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>organización internacional; gobierno local</t>
+          <t>gobierno nacional</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -3388,14 +3556,10 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Internacional</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Voz a Texto; NLP; LLM</t>
-        </is>
-      </c>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3405,22 +3569,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Gaitana IA (resguardo Zenú, Bajo Sinú, Córdoba)</t>
+          <t>ECHO – HáblameD Medellín</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>DUDA(lean SI)</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Presupuestos Participativos; Gobernanza Colaborativa</t>
+          <t>Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Análisis; Traducción Política</t>
+          <t>Implementación; Análisis</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -3428,22 +3592,22 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>sociedad civil</t>
+          <t>organización internacional; gobierno local</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil</t>
+          <t>Gobierno</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>LLM; NLP</t>
+          <t>Voz a Texto; NLP; LLM</t>
         </is>
       </c>
     </row>
@@ -3455,22 +3619,22 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Tenemos que hablar de Colombia</t>
+          <t>Gaitana IA (resguardo Zenú, Bajo Sinú, Córdoba)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>DUDA(lean SI)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
+          <t>Presupuestos Participativos; Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Análisis</t>
+          <t>Análisis; Traducción Política</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
@@ -3478,7 +3642,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>universidad; empresa; sociedad civil</t>
+          <t>sociedad civil</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -3493,19 +3657,19 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>NLP - Tópicos; NLP - Sentiment</t>
+          <t>LLM; NLP</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>U-Report Costa Rica – chatbot juvenil</t>
+          <t>Tenemos que hablar de Colombia</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -3515,7 +3679,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Participación Digital</t>
+          <t>Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3528,34 +3692,34 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>organización internacional</t>
+          <t>universidad; empresa; sociedad civil</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil; Privado</t>
+          <t>Sociedad Civil</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>NLP</t>
+          <t>NLP - Tópicos; NLP - Sentiment</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAGA IA </t>
+          <t>U-Report Costa Rica – chatbot juvenil</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -3565,12 +3729,12 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Referendos e Iniciativas Populares</t>
+          <t>Participación Digital</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
@@ -3578,39 +3742,39 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>gobierno nacional; sociedad civil</t>
+          <t>organización internacional</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil</t>
+          <t>Sociedad Civil; Privado</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>LLM</t>
+          <t>NLP</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guatemala Joven Conversa </t>
+          <t>CiudadanIA</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SI*</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3628,34 +3792,34 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>organización internacional; sociedad civil</t>
+          <t>empresa; universidad; gobierno nacional</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Gobierno</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>NLP - Sentiment; NLP - Tópicos</t>
+          <t>Sistemas de recomendación; LLM</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>HN</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RedPública + iVerify </t>
+          <t xml:space="preserve">PAGA IA </t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -3670,7 +3834,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Análisis</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -3678,34 +3842,34 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>organización internacional; universidad</t>
+          <t>gobierno nacional; sociedad civil</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Gobierno; Academia</t>
+          <t>Sociedad Civil</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Internacional, Nacional</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>NLP - Tópicos</t>
+          <t>LLM</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
+          <t xml:space="preserve">Guatemala Joven Conversa </t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3715,12 +3879,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa; Participación Digital</t>
+          <t>Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Análisis</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
@@ -3728,7 +3892,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>gobierno local</t>
+          <t>organización internacional; sociedad civil</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -3738,48 +3902,64 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>NLP; Otros(no especificado)</t>
+          <t>NLP - Sentiment; NLP - Tópicos</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>HN</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Jalisco - Consulta ¡Armemos un Plan! (Plan Estatal de Desarrollo y Gobernanza 2024-2030)</t>
+          <t xml:space="preserve">RedPública + iVerify </t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>DUDA(lean NO)</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Participación Digital; Gobernanza Colaborativa</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr"/>
+          <t>Referendos e Iniciativas Populares</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Análisis</t>
+        </is>
+      </c>
       <c r="F33" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>gobierno local</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
+          <t>organización internacional; universidad</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Gobierno; Academia</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Internacional, Nacional</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>NLP - Tópicos</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3789,7 +3969,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto CRECES</t>
+          <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3799,12 +3979,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Presupuestos Participativos</t>
+          <t>Gobernanza Colaborativa; Participación Digital</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -3817,7 +3997,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>Gobierno</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -3827,24 +4007,24 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Chatbot - Inespecífico</t>
+          <t>NLP; Otros(no especificado)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
+          <t>Jalisco - Consulta ¡Armemos un Plan! (Plan Estatal de Desarrollo y Gobernanza 2024-2030)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>DUDA(lean NO)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -3852,40 +4032,28 @@
           <t>Participación Digital; Gobernanza Colaborativa</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Análisis; Traducción Política</t>
-        </is>
-      </c>
+      <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>sociedad civil; gobierno nacional</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>Sociedad Civil</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
+          <t>gobierno local</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
+          <t>Presupuesto CRECES</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3895,12 +4063,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
+          <t>Presupuestos Participativos</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Análisis</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
@@ -3908,7 +4076,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>otra institución pública</t>
+          <t>gobierno local</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3918,60 +4086,202 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>NLP - Tópicos; NLP - Sentiment</t>
+          <t>Chatbot - Inespecífico</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Participación Digital; Gobernanza Colaborativa</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Análisis; Traducción Política</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>sociedad civil; gobierno nacional</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Sociedad Civil</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Gobernanza Colaborativa</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Análisis</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>otra institución pública</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>NLP - Tópicos; NLP - Sentiment</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TT</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Participación Digital; Gobernanza Colaborativa</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>gobierno nacional</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>NLP; Resumen automatico; Clasificacion/agrupacion de texto (capacidad de la plataforma sujeta a plan Premium; activacion NO confirmada en TT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>UY</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Pol.is en el Referéndum Nacional de la LUC (Uruguay) — equipo UdelaR</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Referendos e Iniciativas Populares</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Análisis</t>
         </is>
       </c>
-      <c r="F37" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="F40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>universidad</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Sociedad Civil; Academia</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>Internacional</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>Clustering; ML - Inespecífico</t>
         </is>
@@ -4015,7 +4325,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Preliminar y determinístico, para dimensionar el indicador. El principal es el CENTRAL (36 iniciativas). NO es el número final: sale tras la validación manual (pestaña 2).</t>
+          <t>Preliminar y determinístico, para dimensionar el indicador. El principal es el CENTRAL (39 iniciativas). NO es el número final: sale tras la validación manual (pestaña 2).</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4365,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>36 iniciativas. Saca los 7 confirmados no-participación; MANTIENE la frontera (Chatico, Colab) y todas las DUDAs. Es el escenario principal de esta planilla.</t>
+          <t>39 iniciativas. Saca los 4 confirmados no-participación; MANTIENE la frontera (Chatico, Colab) y todas las DUDAs. Es el escenario principal de esta planilla.</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4377,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>27 iniciativas. Solo los ENTRA firmes: saca además la frontera y las DUDAs sin resolver. Cota inferior.</t>
+          <t>30 iniciativas. Solo los ENTRA firmes: saca además la frontera y las DUDAs sin resolver. Cota inferior.</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4389,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>7 confirmados NO: BR-participact-brasil, CO-descongestion-de-solicitudes-diarias-del, CO-dnp-dialogos-regionales-vinculantes-pnd, CR-diara, DO-ciudadania, PE-sistema-de-computo-con-ia-para-las-elecc, TT-engagett-plataforma-go-vocal</t>
+          <t>4 confirmados NO: BR-participact-brasil, CO-descongestion-de-solicitudes-diarias-del, CR-diara, PE-sistema-de-computo-con-ia-para-las-elecc</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4469,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Prom. regional 25 (media de 20) · prom. 42 entre los 12 países con iniciativas.</t>
+          <t>Prom. regional 28 (media de 20) · prom. 40 entre los 14 países con iniciativas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excluir DO CiudadanIA y CO DNP Diálogos (decisión del equipo)
Tras la investigación, el equipo confirma dejarlos fuera:
- DO CiudadanIA: solo atención/servicio, sin módulo de participación.
- CO DNP Diálogos: análisis manual/cualitativo, sin NLP sobre el contenido.

EXCLUIR sube a 6. Queda solo TT EngageTT en DUDA de revisión (grupo C).
calc_preliminar: central baja a 37 inic (prom regional 26); rango techo 29 /
central 26 / conservador 24.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/calculo_preliminar_ILIA2026.xlsx
+++ b/data/gates/calculo_preliminar_ILIA2026.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -590,16 +590,16 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>81</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -749,19 +749,19 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>26</v>
@@ -773,22 +773,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>1</v>
@@ -797,22 +797,22 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Trinidad y Tobago</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E13" s="5" t="n">
         <v>25</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>24</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>1</v>
@@ -821,88 +821,64 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Trinidad y Tobago</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" s="6" t="n">
         <v>22</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>24</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Promedio (países con iniciativas)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr"/>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Promedio (países con iniciativas)</t>
+          <t>Promedio regional (20 países, 0 si no hay)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr"/>
       <c r="E17" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Promedio regional (20 países, 0 si no hay)</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr"/>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="F18" s="3" t="inlineStr"/>
+        <v>26</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -915,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1074,7 +1050,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>75</v>
@@ -1083,16 +1059,16 @@
         <v>67</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>50</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>2</v>
@@ -1338,12 +1314,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -1356,13 +1332,13 @@
         <v>67</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>1</v>
@@ -1371,37 +1347,37 @@
         <v>2</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>67</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>1</v>
@@ -1410,123 +1386,84 @@
         <v>2</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Trinidad y Tobago</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
         <v>40</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Trinidad y Tobago</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>67</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>36</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K15" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1541,7 +1478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1766,105 +1703,84 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>17</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Trinidad y Tobago</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Trinidad y Tobago</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E15" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1949,13 +1865,13 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -2066,7 +1982,7 @@
         <v>81</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>75</v>
@@ -2201,106 +2117,106 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>26</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Trinidad y Tobago</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Trinidad y Tobago</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Rep. Dominicana</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2314,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3523,7 +3439,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>DNP - Diálogos Regionales Vinculantes (PND 2022-2026)</t>
+          <t>ECHO – HáblameD Medellín</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -3533,12 +3449,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Participación Digital; Mini públicos</t>
+          <t>Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Análisis</t>
+          <t>Implementación; Análisis</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
@@ -3546,7 +3462,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>gobierno nacional</t>
+          <t>organización internacional; gobierno local</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -3556,10 +3472,14 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr"/>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Voz a Texto; NLP; LLM</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3569,22 +3489,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ECHO – HáblameD Medellín</t>
+          <t>Gaitana IA (resguardo Zenú, Bajo Sinú, Córdoba)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>DUDA(lean SI)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
+          <t>Presupuestos Participativos; Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Implementación; Análisis</t>
+          <t>Análisis; Traducción Política</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -3592,22 +3512,22 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>organización internacional; gobierno local</t>
+          <t>sociedad civil</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Gobierno</t>
+          <t>Sociedad Civil</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Voz a Texto; NLP; LLM</t>
+          <t>LLM; NLP</t>
         </is>
       </c>
     </row>
@@ -3619,22 +3539,22 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Gaitana IA (resguardo Zenú, Bajo Sinú, Córdoba)</t>
+          <t>Tenemos que hablar de Colombia</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>DUDA(lean SI)</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Presupuestos Participativos; Gobernanza Colaborativa</t>
+          <t>Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Análisis; Traducción Política</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
@@ -3642,7 +3562,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>sociedad civil</t>
+          <t>universidad; empresa; sociedad civil</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -3657,19 +3577,19 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>LLM; NLP</t>
+          <t>NLP - Tópicos; NLP - Sentiment</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Tenemos que hablar de Colombia</t>
+          <t>U-Report Costa Rica – chatbot juvenil</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -3679,7 +3599,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
+          <t>Participación Digital</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3692,34 +3612,34 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>universidad; empresa; sociedad civil</t>
+          <t>organización internacional</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil</t>
+          <t>Sociedad Civil; Privado</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>NLP - Tópicos; NLP - Sentiment</t>
+          <t>NLP</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>U-Report Costa Rica – chatbot juvenil</t>
+          <t xml:space="preserve">PAGA IA </t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -3729,12 +3649,12 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Participación Digital</t>
+          <t>Referendos e Iniciativas Populares</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Análisis</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
@@ -3742,39 +3662,39 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>organización internacional</t>
+          <t>gobierno nacional; sociedad civil</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil; Privado</t>
+          <t>Sociedad Civil</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>NLP</t>
+          <t>LLM</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CiudadanIA</t>
+          <t xml:space="preserve">Guatemala Joven Conversa </t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>SI*</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3792,34 +3712,34 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>empresa; universidad; gobierno nacional</t>
+          <t>organización internacional; sociedad civil</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>Gobierno</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Sistemas de recomendación; LLM</t>
+          <t>NLP - Sentiment; NLP - Tópicos</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>HN</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAGA IA </t>
+          <t xml:space="preserve">RedPública + iVerify </t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -3834,7 +3754,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -3842,34 +3762,34 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>gobierno nacional; sociedad civil</t>
+          <t>organización internacional; universidad</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil</t>
+          <t>Gobierno; Academia</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Internacional, Nacional</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>LLM</t>
+          <t>NLP - Tópicos</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guatemala Joven Conversa </t>
+          <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3879,12 +3799,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
+          <t>Gobernanza Colaborativa; Participación Digital</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
@@ -3892,7 +3812,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>organización internacional; sociedad civil</t>
+          <t>gobierno local</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -3902,64 +3822,48 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>NLP - Sentiment; NLP - Tópicos</t>
+          <t>NLP; Otros(no especificado)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>HN</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RedPública + iVerify </t>
+          <t>Jalisco - Consulta ¡Armemos un Plan! (Plan Estatal de Desarrollo y Gobernanza 2024-2030)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>DUDA(lean NO)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Referendos e Iniciativas Populares</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Análisis</t>
-        </is>
-      </c>
+          <t>Participación Digital; Gobernanza Colaborativa</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>organización internacional; universidad</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>Gobierno; Academia</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Internacional, Nacional</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>NLP - Tópicos</t>
-        </is>
-      </c>
+          <t>gobierno local</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3969,7 +3873,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
+          <t>Presupuesto CRECES</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3979,12 +3883,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa; Participación Digital</t>
+          <t>Presupuestos Participativos</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Análisis</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -3997,7 +3901,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Gobierno</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -4007,24 +3911,24 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>NLP; Otros(no especificado)</t>
+          <t>Chatbot - Inespecífico</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Jalisco - Consulta ¡Armemos un Plan! (Plan Estatal de Desarrollo y Gobernanza 2024-2030)</t>
+          <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>DUDA(lean NO)</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -4032,28 +3936,40 @@
           <t>Participación Digital; Gobernanza Colaborativa</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Análisis; Traducción Política</t>
+        </is>
+      </c>
       <c r="F35" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>gobierno local</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr"/>
+          <t>sociedad civil; gobierno nacional</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Sociedad Civil</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
       <c r="J35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto CRECES</t>
+          <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -4063,12 +3979,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Presupuestos Participativos</t>
+          <t>Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
@@ -4076,7 +3992,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>gobierno local</t>
+          <t>otra institución pública</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -4086,24 +4002,24 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Chatbot - Inespecífico</t>
+          <t>NLP - Tópicos; NLP - Sentiment</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
+          <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -4116,40 +4032,40 @@
           <t>Participación Digital; Gobernanza Colaborativa</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Análisis; Traducción Política</t>
-        </is>
-      </c>
+      <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>sociedad civil; gobierno nacional</t>
+          <t>gobierno nacional</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr"/>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>NLP; Resumen automatico; Clasificacion/agrupacion de texto (capacidad de la plataforma sujeta a plan Premium; activacion NO confirmada en TT)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>UY</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
+          <t>Pol.is en el Referéndum Nacional de la LUC (Uruguay) — equipo UdelaR</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -4159,7 +4075,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
+          <t>Referendos e Iniciativas Populares</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -4172,12 +4088,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>otra institución pública</t>
+          <t>universidad</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>Sociedad Civil; Academia</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -4186,102 +4102,6 @@
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>NLP - Tópicos; NLP - Sentiment</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>TT</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>Participación Digital; Gobernanza Colaborativa</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>gobierno nacional</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>Privado</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>Internacional</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>NLP; Resumen automatico; Clasificacion/agrupacion de texto (capacidad de la plataforma sujeta a plan Premium; activacion NO confirmada en TT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>UY</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Pol.is en el Referéndum Nacional de la LUC (Uruguay) — equipo UdelaR</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Referendos e Iniciativas Populares</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Análisis</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>universidad</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>Sociedad Civil; Academia</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>Internacional</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>Clustering; ML - Inespecífico</t>
         </is>
@@ -4325,7 +4145,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Preliminar y determinístico, para dimensionar el indicador. El principal es el CENTRAL (39 iniciativas). NO es el número final: sale tras la validación manual (pestaña 2).</t>
+          <t>Preliminar y determinístico, para dimensionar el indicador. El principal es el CENTRAL (37 iniciativas). NO es el número final: sale tras la validación manual (pestaña 2).</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4185,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>39 iniciativas. Saca los 4 confirmados no-participación; MANTIENE la frontera (Chatico, Colab) y todas las DUDAs. Es el escenario principal de esta planilla.</t>
+          <t>37 iniciativas. Saca los 6 confirmados no-participación; MANTIENE la frontera (Chatico, Colab) y todas las DUDAs. Es el escenario principal de esta planilla.</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4209,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>4 confirmados NO: BR-participact-brasil, CO-descongestion-de-solicitudes-diarias-del, CR-diara, PE-sistema-de-computo-con-ia-para-las-elecc</t>
+          <t>6 confirmados NO: BR-participact-brasil, CO-descongestion-de-solicitudes-diarias-del, CO-dnp-dialogos-regionales-vinculantes-pnd, CR-diara, DO-ciudadania, PE-sistema-de-computo-con-ia-para-las-elecc</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4289,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Prom. regional 28 (media de 20) · prom. 40 entre los 14 países con iniciativas.</t>
+          <t>Prom. regional 26 (media de 20) · prom. 41 entre los 13 países con iniciativas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BR Colab confirmado ENTRA (módulos de participación: ideas + voto municipal)
Decisión del equipo: Colab permite sugerir ideas y votar en decisiones
municipales, por lo que entra (mismo criterio que Chatico). REVISAR_ENTRA
queda vacío. Rescatados→ENTRA sube a 8; conservador sube a 31 iniciativas.

Queda solo U-Report (CR) en DUDA de frontera, bajo investigación.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/calculo_preliminar_ILIA2026.xlsx
+++ b/data/gates/calculo_preliminar_ILIA2026.xlsx
@@ -1886,7 +1886,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>24</v>
@@ -1964,7 +1964,7 @@
         <v>81</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>30 iniciativas. Solo los ENTRA firmes: saca además la frontera y las DUDAs sin resolver. Cota inferior.</t>
+          <t>31 iniciativas. Solo los ENTRA firmes: saca además la frontera y las DUDAs sin resolver. Cota inferior.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
TT EngageTT → ENTRA (apoyo a la implementación) + doc de casos frontera
- TT EngageTT entra: el chatbot AskNDTS (IA) apoya la implementación del proceso
  NDTS y el módulo Go Vocal Sensemaking está planeado. Rescatados→ENTRA=9;
  DUDA-revisar queda vacío; conservador sube a 32 inic.
- Nuevo data/gates/casos_frontera_ILIA2026.md: documenta los casos borde
  (entraron/salieron/en revisión) y el principio de re-revisión anual, como
  insumo para el reporte final del CENIA.

Queda solo U-Report (CR) pendiente, bajo investigación.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/calculo_preliminar_ILIA2026.xlsx
+++ b/data/gates/calculo_preliminar_ILIA2026.xlsx
@@ -1886,13 +1886,13 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5">
@@ -2174,7 +2174,7 @@
         <v>24</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>31 iniciativas. Solo los ENTRA firmes: saca además la frontera y las DUDAs sin resolver. Cota inferior.</t>
+          <t>32 iniciativas. Solo los ENTRA firmes: saca además la frontera y las DUDAs sin resolver. Cota inferior.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CR U-Report → fuera (encuestas de opinión, no proceso participativo)
Investigación: UNICEF define U-Report como 'encuestas de opinión' (panel de
sondeo/percepción juvenil anónimo); sin proceso participativo estructurado con
incidencia concreta. Por la regla 'solo opinión = fuera' → excluido.

Con esto se resuelven TODOS los casos frontera del ciclo. EXCLUIR=7; sin DUDAs
de frontera pendientes. Guía y doc de casos frontera actualizados.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/calculo_preliminar_ILIA2026.xlsx
+++ b/data/gates/calculo_preliminar_ILIA2026.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -677,22 +677,22 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>BO</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Costa Rica</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>1</v>
@@ -701,19 +701,19 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>28</v>
@@ -725,22 +725,22 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>21</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>1</v>
@@ -749,22 +749,22 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>1</v>
@@ -773,22 +773,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Trinidad y Tobago</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" s="5" t="n">
         <v>25</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>24</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>1</v>
@@ -797,88 +797,64 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Trinidad y Tobago</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" s="6" t="n">
         <v>22</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>24</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Promedio (países con iniciativas)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr"/>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Promedio (países con iniciativas)</t>
+          <t>Promedio regional (20 países, 0 si no hay)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr"/>
       <c r="D16" s="3" t="inlineStr"/>
       <c r="E16" s="5" t="n">
-        <v>41</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Promedio regional (20 países, 0 si no hay)</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="5" t="n">
-        <v>26</v>
-      </c>
-      <c r="F17" s="3" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -891,7 +867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1197,31 +1173,31 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>BO</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Costa Rica</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>67</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>1</v>
@@ -1230,37 +1206,37 @@
         <v>2</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
         <v>20</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>67</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>1</v>
@@ -1275,12 +1251,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
@@ -1293,13 +1269,13 @@
         <v>67</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1</v>
@@ -1308,37 +1284,37 @@
         <v>2</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>67</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>1</v>
@@ -1347,123 +1323,84 @@
         <v>2</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Trinidad y Tobago</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
         <v>40</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Trinidad y Tobago</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>67</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>36</v>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="H14" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="I14" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K14" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1478,7 +1415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1640,54 +1577,54 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>BO</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Costa Rica</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>8</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
         <v>25</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
@@ -1703,84 +1640,63 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Trinidad y Tobago</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Trinidad y Tobago</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E14" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1865,13 +1781,13 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
@@ -2054,33 +1970,33 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>BO</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Costa Rica</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
@@ -2096,106 +2012,106 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Panamá</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Trinidad y Tobago</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Trinidad y Tobago</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Costa Rica</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -2230,7 +2146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3584,12 +3500,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>U-Report Costa Rica – chatbot juvenil</t>
+          <t xml:space="preserve">PAGA IA </t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -3599,12 +3515,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Participación Digital</t>
+          <t>Referendos e Iniciativas Populares</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Análisis</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
@@ -3612,34 +3528,34 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>organización internacional</t>
+          <t>gobierno nacional; sociedad civil</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil; Privado</t>
+          <t>Sociedad Civil</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>NLP</t>
+          <t>LLM</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAGA IA </t>
+          <t xml:space="preserve">Guatemala Joven Conversa </t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -3649,7 +3565,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Referendos e Iniciativas Populares</t>
+          <t>Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -3662,34 +3578,34 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>gobierno nacional; sociedad civil</t>
+          <t>organización internacional; sociedad civil</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil</t>
+          <t>Gobierno</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>LLM</t>
+          <t>NLP - Sentiment; NLP - Tópicos</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>HN</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guatemala Joven Conversa </t>
+          <t xml:space="preserve">RedPública + iVerify </t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -3699,12 +3615,12 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
+          <t>Referendos e Iniciativas Populares</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
@@ -3712,34 +3628,34 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>organización internacional; sociedad civil</t>
+          <t>organización internacional; universidad</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Gobierno</t>
+          <t>Gobierno; Academia</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Internacional, Nacional</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>NLP - Sentiment; NLP - Tópicos</t>
+          <t>NLP - Tópicos</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>HN</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RedPública + iVerify </t>
+          <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -3749,7 +3665,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Referendos e Iniciativas Populares</t>
+          <t>Gobernanza Colaborativa; Participación Digital</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -3762,22 +3678,22 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>organización internacional; universidad</t>
+          <t>gobierno local</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Gobierno; Academia</t>
+          <t>Gobierno</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Internacional, Nacional</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>NLP - Tópicos</t>
+          <t>NLP; Otros(no especificado)</t>
         </is>
       </c>
     </row>
@@ -3789,47 +3705,31 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
+          <t>Jalisco - Consulta ¡Armemos un Plan! (Plan Estatal de Desarrollo y Gobernanza 2024-2030)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>DUDA(lean NO)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa; Participación Digital</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Análisis</t>
-        </is>
-      </c>
+          <t>Participación Digital; Gobernanza Colaborativa</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
           <t>gobierno local</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Gobierno</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>NLP; Otros(no especificado)</t>
-        </is>
-      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3839,41 +3739,57 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Jalisco - Consulta ¡Armemos un Plan! (Plan Estatal de Desarrollo y Gobernanza 2024-2030)</t>
+          <t>Presupuesto CRECES</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>DUDA(lean NO)</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Participación Digital; Gobernanza Colaborativa</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr"/>
+          <t>Presupuestos Participativos</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Implementación</t>
+        </is>
+      </c>
       <c r="F33" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
           <t>gobierno local</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Chatbot - Inespecífico</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto CRECES</t>
+          <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3883,12 +3799,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Presupuestos Participativos</t>
+          <t>Participación Digital; Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Análisis; Traducción Política</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -3896,12 +3812,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>gobierno local</t>
+          <t>sociedad civil; gobierno nacional</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>Sociedad Civil</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -3909,21 +3825,17 @@
           <t>Nacional</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>Chatbot - Inespecífico</t>
-        </is>
-      </c>
+      <c r="J34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
+          <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3933,12 +3845,12 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Participación Digital; Gobernanza Colaborativa</t>
+          <t>Gobernanza Colaborativa</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Análisis; Traducción Política</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
@@ -3946,30 +3858,34 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>sociedad civil; gobierno nacional</t>
+          <t>otra institución pública</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Sociedad Civil</t>
+          <t>Privado</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr"/>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>NLP - Tópicos; NLP - Sentiment</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
+          <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3979,20 +3895,16 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Análisis</t>
-        </is>
-      </c>
+          <t>Participación Digital; Gobernanza Colaborativa</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>otra institución pública</t>
+          <t>gobierno nacional</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -4007,19 +3919,19 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>NLP - Tópicos; NLP - Sentiment</t>
+          <t>NLP; Resumen automatico; Clasificacion/agrupacion de texto (capacidad de la plataforma sujeta a plan Premium; activacion NO confirmada en TT)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>UY</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
+          <t>Pol.is en el Referéndum Nacional de la LUC (Uruguay) — equipo UdelaR</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -4029,21 +3941,25 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Participación Digital; Gobernanza Colaborativa</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr"/>
+          <t>Referendos e Iniciativas Populares</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Análisis</t>
+        </is>
+      </c>
       <c r="F37" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>gobierno nacional</t>
+          <t>universidad</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>Sociedad Civil; Academia</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -4052,56 +3968,6 @@
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>NLP; Resumen automatico; Clasificacion/agrupacion de texto (capacidad de la plataforma sujeta a plan Premium; activacion NO confirmada en TT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>UY</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Pol.is en el Referéndum Nacional de la LUC (Uruguay) — equipo UdelaR</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Referendos e Iniciativas Populares</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Análisis</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>universidad</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Sociedad Civil; Academia</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>Internacional</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>Clustering; ML - Inespecífico</t>
         </is>
@@ -4145,7 +4011,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Preliminar y determinístico, para dimensionar el indicador. El principal es el CENTRAL (37 iniciativas). NO es el número final: sale tras la validación manual (pestaña 2).</t>
+          <t>Preliminar y determinístico, para dimensionar el indicador. El principal es el CENTRAL (36 iniciativas). NO es el número final: sale tras la validación manual (pestaña 2).</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4051,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>37 iniciativas. Saca los 6 confirmados no-participación; MANTIENE la frontera (Chatico, Colab) y todas las DUDAs. Es el escenario principal de esta planilla.</t>
+          <t>36 iniciativas. Saca los 7 confirmados no-participación; MANTIENE la frontera (Chatico, Colab) y todas las DUDAs. Es el escenario principal de esta planilla.</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4075,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>6 confirmados NO: BR-participact-brasil, CO-descongestion-de-solicitudes-diarias-del, CO-dnp-dialogos-regionales-vinculantes-pnd, CR-diara, DO-ciudadania, PE-sistema-de-computo-con-ia-para-las-elecc</t>
+          <t>7 confirmados NO: BR-participact-brasil, CO-descongestion-de-solicitudes-diarias-del, CO-dnp-dialogos-regionales-vinculantes-pnd, CR-diara, CR-u-report-costa-rica-chatbot-juvenil, DO-ciudadania, PE-sistema-de-computo-con-ia-para-las-elecc</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4155,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Prom. regional 26 (media de 20) · prom. 41 entre los 13 países con iniciativas.</t>
+          <t>Prom. regional 25 (media de 20) · prom. 42 entre los 12 países con iniciativas.</t>
         </is>
       </c>
     </row>

</xml_diff>